<commit_message>
Clarify fresh glossary export step in template
</commit_message>
<xml_diff>
--- a/assets/glossary-template.xlsx
+++ b/assets/glossary-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="詞彙校正" sheetId="1" r:id="R9b7364d03c5e4803"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="背景與規則" sheetId="2" r:id="Rcf46ab63948848b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="詞彙校正" sheetId="1" r:id="Ra4886a5312ef429f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="背景與規則" sheetId="2" r:id="R7a0bfd277de4423b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -113,7 +113,7 @@
         <x:color rgb="FF737C8A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF0F4"/>
         </x:patternFill>
       </x:fill>
@@ -124,7 +124,7 @@
         <x:color rgb="FF6E4C13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0BD"/>
         </x:patternFill>
       </x:fill>
@@ -134,7 +134,7 @@
         <x:color rgb="FF737C8A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF0F4"/>
         </x:patternFill>
       </x:fill>
@@ -363,7 +363,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>每次修改後儲存；重新整理錄音時會讀取新版。</x:v>
+        <x:v>修改後請匯出最新版 Excel；重新整理錄音時選擇該檔案。</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>

</xml_diff>